<commit_message>
Add Map and Update Admin Page
</commit_message>
<xml_diff>
--- a/exports/sales_data.xlsx
+++ b/exports/sales_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="214">
   <si>
     <t>Order ID</t>
   </si>
@@ -286,6 +286,21 @@
     <t>2026-05-01T14:51:54.558Z</t>
   </si>
   <si>
+    <t>ATH3323452364</t>
+  </si>
+  <si>
+    <t>2026-05-03T18:33:54.528Z</t>
+  </si>
+  <si>
+    <t>2026-05-03T18:34:34.153Z</t>
+  </si>
+  <si>
+    <t>ATH3685738410</t>
+  </si>
+  <si>
+    <t>2026-05-03T19:34:17.398Z</t>
+  </si>
+  <si>
     <t>Customer ID</t>
   </si>
   <si>
@@ -361,7 +376,7 @@
     <t>69df56a29a28b213c15d5c44</t>
   </si>
   <si>
-    <t>2026-05-01T14:50:30.330Z</t>
+    <t>2026-05-03T19:34:18.614Z</t>
   </si>
   <si>
     <t>Product ID</t>
@@ -391,12 +406,12 @@
     <t>69d8ef144922394efe9aede2</t>
   </si>
   <si>
+    <t>69d8ef254922394efe9aedfe</t>
+  </si>
+  <si>
     <t>Low</t>
   </si>
   <si>
-    <t>69d8ef254922394efe9aedfe</t>
-  </si>
-  <si>
     <t>69d8ef134922394efe9aede0</t>
   </si>
   <si>
@@ -598,6 +613,15 @@
     <t>2026-04-29T13:58:16.464Z</t>
   </si>
   <si>
+    <t>69f89d51987705d82e7eeaef</t>
+  </si>
+  <si>
+    <t>roro</t>
+  </si>
+  <si>
+    <t>2026-05-04T13:21:20.906Z</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -629,6 +653,9 @@
   </si>
   <si>
     <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-03</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -1967,6 +1994,88 @@
       </c>
       <c r="M23" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>120</v>
+      </c>
+      <c r="I24">
+        <v>120</v>
+      </c>
+      <c r="J24" t="s">
+        <v>41</v>
+      </c>
+      <c r="K24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L24" t="s">
+        <v>91</v>
+      </c>
+      <c r="M24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>120</v>
+      </c>
+      <c r="I25">
+        <v>120</v>
+      </c>
+      <c r="J25" t="s">
+        <v>85</v>
+      </c>
+      <c r="K25" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" t="s">
+        <v>94</v>
+      </c>
+      <c r="M25" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1991,39 +2100,39 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -2044,13 +2153,13 @@
         <v>78</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I2" t="s">
         <v>26</v>
       </c>
       <c r="J2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -2082,7 +2191,7 @@
         <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -2114,21 +2223,21 @@
         <v>18</v>
       </c>
       <c r="J4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D5" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2146,21 +2255,21 @@
         <v>15</v>
       </c>
       <c r="J5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -2178,44 +2287,44 @@
         <v>15</v>
       </c>
       <c r="J6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" t="s">
         <v>113</v>
-      </c>
-      <c r="D7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s">
         <v>38</v>
@@ -2227,22 +2336,22 @@
         <v>40</v>
       </c>
       <c r="E8">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F8">
-        <v>1572</v>
+        <v>1852</v>
       </c>
       <c r="G8" t="s">
         <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I8" t="s">
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2253,7 +2362,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2266,7 +2375,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
@@ -2275,24 +2384,24 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -2313,12 +2422,12 @@
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B3" t="s">
         <v>25</v>
@@ -2327,24 +2436,24 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>480</v>
+        <v>720</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
@@ -2365,12 +2474,12 @@
         <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
@@ -2391,12 +2500,12 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B6" t="s">
         <v>55</v>
@@ -2417,12 +2526,12 @@
         <v>15</v>
       </c>
       <c r="H6" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
@@ -2443,12 +2552,12 @@
         <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
@@ -2469,12 +2578,12 @@
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
         <v>80</v>
@@ -2495,12 +2604,12 @@
         <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B10" t="s">
         <v>59</v>
@@ -2521,15 +2630,15 @@
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C11" t="s">
         <v>60</v>
@@ -2547,15 +2656,15 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C12" t="s">
         <v>23</v>
@@ -2573,15 +2682,15 @@
         <v>15</v>
       </c>
       <c r="H12" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
@@ -2599,15 +2708,15 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C14" t="s">
         <v>60</v>
@@ -2625,15 +2734,15 @@
         <v>15</v>
       </c>
       <c r="H14" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
@@ -2651,15 +2760,15 @@
         <v>15</v>
       </c>
       <c r="H15" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B16" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
@@ -2677,15 +2786,15 @@
         <v>15</v>
       </c>
       <c r="H16" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B17" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
@@ -2703,15 +2812,15 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
@@ -2729,18 +2838,18 @@
         <v>15</v>
       </c>
       <c r="H18" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C19" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D19">
         <v>5</v>
@@ -2755,18 +2864,18 @@
         <v>15</v>
       </c>
       <c r="H19" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B20" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C20" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -2781,18 +2890,18 @@
         <v>15</v>
       </c>
       <c r="H20" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B21" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C21" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D21">
         <v>4</v>
@@ -2807,15 +2916,15 @@
         <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B22" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C22" t="s">
         <v>29</v>
@@ -2833,15 +2942,15 @@
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B23" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -2859,15 +2968,15 @@
         <v>15</v>
       </c>
       <c r="H23" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B24" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C24" t="s">
         <v>26</v>
@@ -2885,15 +2994,15 @@
         <v>15</v>
       </c>
       <c r="H24" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B25" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C25" t="s">
         <v>23</v>
@@ -2911,15 +3020,15 @@
         <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B26" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C26" t="s">
         <v>23</v>
@@ -2937,15 +3046,15 @@
         <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B27" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C27" t="s">
         <v>23</v>
@@ -2963,15 +3072,15 @@
         <v>15</v>
       </c>
       <c r="H27" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B28" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C28" t="s">
         <v>23</v>
@@ -2989,15 +3098,15 @@
         <v>15</v>
       </c>
       <c r="H28" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B29" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C29" t="s">
         <v>23</v>
@@ -3015,15 +3124,15 @@
         <v>15</v>
       </c>
       <c r="H29" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C30" t="s">
         <v>60</v>
@@ -3041,15 +3150,15 @@
         <v>15</v>
       </c>
       <c r="H30" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B31" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C31" t="s">
         <v>29</v>
@@ -3067,15 +3176,15 @@
         <v>15</v>
       </c>
       <c r="H31" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B32" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C32" t="s">
         <v>18</v>
@@ -3093,15 +3202,15 @@
         <v>15</v>
       </c>
       <c r="H32" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B33" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C33" t="s">
         <v>29</v>
@@ -3119,15 +3228,15 @@
         <v>15</v>
       </c>
       <c r="H33" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B34" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C34" t="s">
         <v>29</v>
@@ -3145,15 +3254,15 @@
         <v>15</v>
       </c>
       <c r="H34" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B35" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C35" t="s">
         <v>60</v>
@@ -3171,15 +3280,15 @@
         <v>15</v>
       </c>
       <c r="H35" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B36" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C36" t="s">
         <v>23</v>
@@ -3197,15 +3306,15 @@
         <v>15</v>
       </c>
       <c r="H36" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B37" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C37" t="s">
         <v>26</v>
@@ -3223,15 +3332,15 @@
         <v>15</v>
       </c>
       <c r="H37" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B38" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C38" t="s">
         <v>23</v>
@@ -3249,18 +3358,18 @@
         <v>15</v>
       </c>
       <c r="H38" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B39" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C39" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D39">
         <v>20</v>
@@ -3272,10 +3381,36 @@
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="H39" t="s">
-        <v>131</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>199</v>
+      </c>
+      <c r="B40" t="s">
+        <v>200</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40">
+        <v>20</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40" t="s">
+        <v>201</v>
+      </c>
+      <c r="H40" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3286,7 +3421,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -3297,30 +3432,30 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B2">
         <v>464</v>
@@ -3343,7 +3478,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B3">
         <v>630</v>
@@ -3366,7 +3501,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B4">
         <v>1553</v>
@@ -3389,7 +3524,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B5">
         <v>64</v>
@@ -3412,7 +3547,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B6">
         <v>140</v>
@@ -3435,7 +3570,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B7">
         <v>170</v>
@@ -3454,6 +3589,29 @@
       </c>
       <c r="G7">
         <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B8">
+        <v>280</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update the Delivery Page
</commit_message>
<xml_diff>
--- a/exports/sales_data.xlsx
+++ b/exports/sales_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="271">
   <si>
     <t>Order ID</t>
   </si>
@@ -451,6 +451,21 @@
     <t>2026-05-04T22:10:40.162Z</t>
   </si>
   <si>
+    <t>ATH7817978342</t>
+  </si>
+  <si>
+    <t>2026-05-06T14:36:19.786Z</t>
+  </si>
+  <si>
+    <t>2026-05-06T14:39:38.351Z</t>
+  </si>
+  <si>
+    <t>ATH9038552316</t>
+  </si>
+  <si>
+    <t>2026-05-06T17:59:45.550Z</t>
+  </si>
+  <si>
     <t>Customer ID</t>
   </si>
   <si>
@@ -484,15 +499,15 @@
     <t>69df51939a28b213c15d5bfb</t>
   </si>
   <si>
-    <t>2026-04-28T12:17:31.160Z</t>
+    <t>2026-05-06T17:59:46.019Z</t>
+  </si>
+  <si>
+    <t>VIP</t>
   </si>
   <si>
     <t>Regular</t>
   </si>
   <si>
-    <t>VIP</t>
-  </si>
-  <si>
     <t>69d8d572ae6a1e8c2c032bc2</t>
   </si>
   <si>
@@ -550,16 +565,28 @@
     <t>69d8ef134922394efe9aeddf</t>
   </si>
   <si>
-    <t>Out of Stock</t>
+    <t>2026-05-06T15:21:31.177Z</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
   <si>
     <t>69d8ef144922394efe9aede2</t>
   </si>
   <si>
+    <t>2026-05-06T15:21:02.483Z</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
     <t>69d8ef134922394efe9aede0</t>
   </si>
   <si>
-    <t>Critical</t>
+    <t>2026-05-06T15:21:18.409Z</t>
+  </si>
+  <si>
+    <t>Low</t>
   </si>
   <si>
     <t>69d8ef284922394efe9aee03</t>
@@ -571,21 +598,18 @@
     <t>69d8ef1d4922394efe9aedf1</t>
   </si>
   <si>
+    <t>2026-05-06T15:29:56.291Z</t>
+  </si>
+  <si>
     <t>69d8ef254922394efe9aedfe</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>69d8ef144922394efe9aede1</t>
   </si>
   <si>
     <t>69d8ef264922394efe9aee00</t>
   </si>
   <si>
-    <t>OK</t>
-  </si>
-  <si>
     <t>69d8ef174922394efe9aede7</t>
   </si>
   <si>
@@ -800,6 +824,9 @@
   </si>
   <si>
     <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -3153,7 +3180,7 @@
         <v>94</v>
       </c>
       <c r="J48" t="s">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="K48" t="s">
         <v>20</v>
@@ -3162,6 +3189,88 @@
         <v>144</v>
       </c>
       <c r="M48" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>145</v>
+      </c>
+      <c r="B49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" t="s">
+        <v>77</v>
+      </c>
+      <c r="D49" t="s">
+        <v>31</v>
+      </c>
+      <c r="E49" t="s">
+        <v>124</v>
+      </c>
+      <c r="F49" t="s">
+        <v>60</v>
+      </c>
+      <c r="G49">
+        <v>1</v>
+      </c>
+      <c r="H49">
+        <v>50</v>
+      </c>
+      <c r="I49">
+        <v>50</v>
+      </c>
+      <c r="J49" t="s">
+        <v>41</v>
+      </c>
+      <c r="K49" t="s">
+        <v>20</v>
+      </c>
+      <c r="L49" t="s">
+        <v>146</v>
+      </c>
+      <c r="M49" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>148</v>
+      </c>
+      <c r="B50" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" t="s">
+        <v>77</v>
+      </c>
+      <c r="D50" t="s">
+        <v>31</v>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+      <c r="F50" t="s">
+        <v>18</v>
+      </c>
+      <c r="G50">
+        <v>8</v>
+      </c>
+      <c r="H50">
+        <v>150</v>
+      </c>
+      <c r="I50">
+        <v>1200</v>
+      </c>
+      <c r="J50" t="s">
+        <v>85</v>
+      </c>
+      <c r="K50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L50" t="s">
+        <v>149</v>
+      </c>
+      <c r="M50" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3187,39 +3296,39 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -3231,22 +3340,22 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>355</v>
+        <v>1645</v>
       </c>
       <c r="G2" t="s">
         <v>78</v>
       </c>
       <c r="H2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -3278,7 +3387,7 @@
         <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -3310,21 +3419,21 @@
         <v>18</v>
       </c>
       <c r="J4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D5" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3342,21 +3451,21 @@
         <v>15</v>
       </c>
       <c r="J5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C6" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -3374,44 +3483,44 @@
         <v>15</v>
       </c>
       <c r="J6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B7" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" t="s">
         <v>168</v>
-      </c>
-      <c r="D7" t="s">
-        <v>166</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B8" t="s">
         <v>38</v>
@@ -3432,13 +3541,13 @@
         <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="I8" t="s">
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -3462,7 +3571,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
@@ -3471,24 +3580,24 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -3497,24 +3606,24 @@
         <v>18</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E2">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F2">
-        <v>1950</v>
+        <v>3150</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>183</v>
       </c>
       <c r="H2" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B3" t="s">
         <v>25</v>
@@ -3523,7 +3632,7 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>9</v>
@@ -3532,15 +3641,15 @@
         <v>1080</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>186</v>
       </c>
       <c r="H3" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B4" t="s">
         <v>28</v>
@@ -3549,7 +3658,7 @@
         <v>29</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4">
         <v>10</v>
@@ -3558,15 +3667,15 @@
         <v>600</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>189</v>
       </c>
       <c r="H4" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
@@ -3587,12 +3696,12 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="B6" t="s">
         <v>116</v>
@@ -3613,12 +3722,12 @@
         <v>15</v>
       </c>
       <c r="H6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B7" t="s">
         <v>55</v>
@@ -3627,7 +3736,7 @@
         <v>23</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -3636,15 +3745,15 @@
         <v>285</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>194</v>
       </c>
       <c r="H7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="B8" t="s">
         <v>48</v>
@@ -3665,12 +3774,12 @@
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B9" t="s">
         <v>124</v>
@@ -3679,24 +3788,24 @@
         <v>60</v>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
@@ -3717,12 +3826,12 @@
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B11" t="s">
         <v>80</v>
@@ -3743,12 +3852,12 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B12" t="s">
         <v>59</v>
@@ -3769,12 +3878,12 @@
         <v>15</v>
       </c>
       <c r="H12" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B13" t="s">
         <v>139</v>
@@ -3795,15 +3904,15 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="C14" t="s">
         <v>23</v>
@@ -3821,15 +3930,15 @@
         <v>15</v>
       </c>
       <c r="H14" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B15" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
@@ -3847,15 +3956,15 @@
         <v>15</v>
       </c>
       <c r="H15" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B16" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
@@ -3873,15 +3982,15 @@
         <v>15</v>
       </c>
       <c r="H16" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B17" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
@@ -3899,15 +4008,15 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B18" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C18" t="s">
         <v>18</v>
@@ -3925,15 +4034,15 @@
         <v>15</v>
       </c>
       <c r="H18" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B19" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
@@ -3951,15 +4060,15 @@
         <v>15</v>
       </c>
       <c r="H19" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B20" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -3977,15 +4086,15 @@
         <v>15</v>
       </c>
       <c r="H20" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B21" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C21" t="s">
         <v>117</v>
@@ -4003,15 +4112,15 @@
         <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B22" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="C22" t="s">
         <v>117</v>
@@ -4029,15 +4138,15 @@
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B23" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -4055,15 +4164,15 @@
         <v>15</v>
       </c>
       <c r="H23" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B24" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C24" t="s">
         <v>29</v>
@@ -4081,15 +4190,15 @@
         <v>15</v>
       </c>
       <c r="H24" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B25" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="C25" t="s">
         <v>26</v>
@@ -4107,15 +4216,15 @@
         <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B26" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="C26" t="s">
         <v>23</v>
@@ -4133,15 +4242,15 @@
         <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B27" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C27" t="s">
         <v>23</v>
@@ -4159,15 +4268,15 @@
         <v>15</v>
       </c>
       <c r="H27" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B28" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="C28" t="s">
         <v>23</v>
@@ -4185,15 +4294,15 @@
         <v>15</v>
       </c>
       <c r="H28" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C29" t="s">
         <v>23</v>
@@ -4211,15 +4320,15 @@
         <v>15</v>
       </c>
       <c r="H29" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B30" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="C30" t="s">
         <v>23</v>
@@ -4237,15 +4346,15 @@
         <v>15</v>
       </c>
       <c r="H30" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B31" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="C31" t="s">
         <v>60</v>
@@ -4263,15 +4372,15 @@
         <v>15</v>
       </c>
       <c r="H31" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B32" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C32" t="s">
         <v>18</v>
@@ -4289,15 +4398,15 @@
         <v>15</v>
       </c>
       <c r="H32" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B33" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="C33" t="s">
         <v>29</v>
@@ -4315,15 +4424,15 @@
         <v>15</v>
       </c>
       <c r="H33" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B34" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="C34" t="s">
         <v>29</v>
@@ -4341,15 +4450,15 @@
         <v>15</v>
       </c>
       <c r="H34" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B35" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C35" t="s">
         <v>60</v>
@@ -4367,15 +4476,15 @@
         <v>15</v>
       </c>
       <c r="H35" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B36" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="C36" t="s">
         <v>23</v>
@@ -4393,15 +4502,15 @@
         <v>15</v>
       </c>
       <c r="H36" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B37" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="C37" t="s">
         <v>26</v>
@@ -4419,15 +4528,15 @@
         <v>15</v>
       </c>
       <c r="H37" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="B38" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="C38" t="s">
         <v>23</v>
@@ -4445,15 +4554,15 @@
         <v>15</v>
       </c>
       <c r="H38" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B39" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="C39" t="s">
         <v>117</v>
@@ -4468,18 +4577,18 @@
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="H39" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B40" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C40" t="s">
         <v>23</v>
@@ -4494,10 +4603,10 @@
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="H40" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -4508,7 +4617,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -4519,30 +4628,30 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B2">
         <v>464</v>
@@ -4565,7 +4674,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B3">
         <v>630</v>
@@ -4588,7 +4697,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B4">
         <v>1553</v>
@@ -4611,7 +4720,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B5">
         <v>64</v>
@@ -4634,7 +4743,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B6">
         <v>140</v>
@@ -4657,7 +4766,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B7">
         <v>170</v>
@@ -4680,7 +4789,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B8">
         <v>280</v>
@@ -4703,7 +4812,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B9">
         <v>2738</v>
@@ -4722,6 +4831,29 @@
       </c>
       <c r="G9">
         <v>119.04</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B10">
+        <v>1290</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10">
+        <v>645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add analystics tools in admine page
</commit_message>
<xml_diff>
--- a/exports/sales_data.xlsx
+++ b/exports/sales_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="333">
   <si>
     <t>Order ID</t>
   </si>
@@ -466,6 +466,9 @@
     <t>2026-05-06T17:59:45.550Z</t>
   </si>
   <si>
+    <t>2026-05-06T18:01:45.395Z</t>
+  </si>
+  <si>
     <t>Customer ID</t>
   </si>
   <si>
@@ -574,24 +577,24 @@
     <t>69d8ef144922394efe9aede2</t>
   </si>
   <si>
-    <t>2026-05-06T15:21:02.483Z</t>
+    <t>2026-05-10T21:40:23.579Z</t>
+  </si>
+  <si>
+    <t>69d8ef134922394efe9aede0</t>
+  </si>
+  <si>
+    <t>2026-05-06T15:21:18.409Z</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>69d8ef284922394efe9aee03</t>
   </si>
   <si>
     <t>Critical</t>
   </si>
   <si>
-    <t>69d8ef134922394efe9aede0</t>
-  </si>
-  <si>
-    <t>2026-05-06T15:21:18.409Z</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>69d8ef284922394efe9aee03</t>
-  </si>
-  <si>
     <t>69d8ef1b4922394efe9aeded</t>
   </si>
   <si>
@@ -785,6 +788,189 @@
   </si>
   <si>
     <t>2026-05-04T13:21:20.906Z</t>
+  </si>
+  <si>
+    <t>69fe61604dfc5e28d4778a0d</t>
+  </si>
+  <si>
+    <t>Athar Midnight Heritage Tote</t>
+  </si>
+  <si>
+    <t>2026-05-08T22:19:11.313Z</t>
+  </si>
+  <si>
+    <t>69ff674c930f43fc7389752d</t>
+  </si>
+  <si>
+    <t>Athar Desert Sand Heritage Tote</t>
+  </si>
+  <si>
+    <t>2026-05-09T16:56:44.466Z</t>
+  </si>
+  <si>
+    <t>69ff827b61b6c73a91e2da68</t>
+  </si>
+  <si>
+    <t>Athar Midnight Heritage Hobo Bag</t>
+  </si>
+  <si>
+    <t>2026-05-09T18:52:43.570Z</t>
+  </si>
+  <si>
+    <t>69ff83cf61b6c73a91e2da6c</t>
+  </si>
+  <si>
+    <t>Athar Pearl Heritage Tote</t>
+  </si>
+  <si>
+    <t>2026-05-09T18:58:23.701Z</t>
+  </si>
+  <si>
+    <t>69ff852f61b6c73a91e2da71</t>
+  </si>
+  <si>
+    <t>Athar Earthly Heritage Bucket Bag</t>
+  </si>
+  <si>
+    <t>2026-05-09T19:04:14.801Z</t>
+  </si>
+  <si>
+    <t>69ff879861b6c73a91e2da75</t>
+  </si>
+  <si>
+    <t>Nablus Tote Bag</t>
+  </si>
+  <si>
+    <t>2026-05-09T19:14:32.698Z</t>
+  </si>
+  <si>
+    <t>69ff891861b6c73a91e2da7a</t>
+  </si>
+  <si>
+    <t>Athar Heritage Box Bag - Nablus Edition.</t>
+  </si>
+  <si>
+    <t>2026-05-09T19:20:55.822Z</t>
+  </si>
+  <si>
+    <t>69ff8a3f61b6c73a91e2da7e</t>
+  </si>
+  <si>
+    <t>Athar Olive Heritage Envelope Bag</t>
+  </si>
+  <si>
+    <t>2026-05-09T19:25:51.651Z</t>
+  </si>
+  <si>
+    <t>69ff8c0061b6c73a91e2da82</t>
+  </si>
+  <si>
+    <t>Title: Athar Burgundy Heritage Top Handle bag</t>
+  </si>
+  <si>
+    <t>2026-05-09T19:33:19.881Z</t>
+  </si>
+  <si>
+    <t>6a002e4bbd1dc81199f3c5f2</t>
+  </si>
+  <si>
+    <t>Athar Crimson Heritage Wallet</t>
+  </si>
+  <si>
+    <t>2026-05-10T07:05:47.340Z</t>
+  </si>
+  <si>
+    <t>6a002f37bd1dc81199f3c5f4</t>
+  </si>
+  <si>
+    <t>Athar Lavender Heritage Wallet</t>
+  </si>
+  <si>
+    <t>2026-05-10T07:09:43.713Z</t>
+  </si>
+  <si>
+    <t>6a002fe7bd1dc81199f3c5f6</t>
+  </si>
+  <si>
+    <t>Athar Olive Grove Wallet</t>
+  </si>
+  <si>
+    <t>2026-05-10T07:12:39.356Z</t>
+  </si>
+  <si>
+    <t>6a003bc8ae90c37e771e5014</t>
+  </si>
+  <si>
+    <t>Athar Slate Heritage Wallet</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:03:20.059Z</t>
+  </si>
+  <si>
+    <t>6a003bc8ae90c37e771e5015</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:03:20.316Z</t>
+  </si>
+  <si>
+    <t>6a003bcaae90c37e771e5017</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:03:21.625Z</t>
+  </si>
+  <si>
+    <t>6a003cafae90c37e771e5019</t>
+  </si>
+  <si>
+    <t>Athar Golden Dome Heritage Watch</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:07:10.984Z</t>
+  </si>
+  <si>
+    <t>6a003d4aae90c37e771e501b</t>
+  </si>
+  <si>
+    <t>Athar Tiberias Golden Mesh Watch</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:09:46.205Z</t>
+  </si>
+  <si>
+    <t>6a003efdae90c37e771e501d</t>
+  </si>
+  <si>
+    <t>The Everlasting Bloom Motif.</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:17:01.304Z</t>
+  </si>
+  <si>
+    <t>6a004120ae90c37e771e501f</t>
+  </si>
+  <si>
+    <t>Athar Jaffa Sunset Watch</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:26:08.316Z</t>
+  </si>
+  <si>
+    <t>6a0041e5ae90c37e771e5021</t>
+  </si>
+  <si>
+    <t>Athar Bethlehem Dove of Peace Watch</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:29:25.686Z</t>
+  </si>
+  <si>
+    <t>6a004302ae90c37e771e5023</t>
+  </si>
+  <si>
+    <t>Athar Ramallah Starry Horizon Watch</t>
+  </si>
+  <si>
+    <t>2026-05-10T08:34:10.136Z</t>
   </si>
   <si>
     <t>Date</t>
@@ -3262,7 +3448,7 @@
         <v>1200</v>
       </c>
       <c r="J50" t="s">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="K50" t="s">
         <v>20</v>
@@ -3271,7 +3457,7 @@
         <v>149</v>
       </c>
       <c r="M50" t="s">
-        <v>15</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3296,39 +3482,39 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -3349,13 +3535,13 @@
         <v>78</v>
       </c>
       <c r="H2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I2" t="s">
         <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -3387,7 +3573,7 @@
         <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -3419,21 +3605,21 @@
         <v>18</v>
       </c>
       <c r="J4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3451,54 +3637,54 @@
         <v>15</v>
       </c>
       <c r="J5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" t="s">
         <v>169</v>
-      </c>
-      <c r="B6" t="s">
-        <v>165</v>
-      </c>
-      <c r="C6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" t="s">
-        <v>171</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D7" t="s">
         <v>172</v>
       </c>
-      <c r="B7" t="s">
-        <v>165</v>
-      </c>
-      <c r="C7" t="s">
-        <v>173</v>
-      </c>
-      <c r="D7" t="s">
-        <v>171</v>
-      </c>
       <c r="E7">
         <v>0</v>
       </c>
@@ -3515,12 +3701,12 @@
         <v>15</v>
       </c>
       <c r="J7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" t="s">
         <v>38</v>
@@ -3541,13 +3727,13 @@
         <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I8" t="s">
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -3558,11 +3744,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="33" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
@@ -3571,7 +3757,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
@@ -3580,24 +3766,24 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -3606,7 +3792,7 @@
         <v>18</v>
       </c>
       <c r="D2">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E2">
         <v>21</v>
@@ -3615,15 +3801,15 @@
         <v>3150</v>
       </c>
       <c r="G2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B3" t="s">
         <v>25</v>
@@ -3632,7 +3818,7 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>137</v>
       </c>
       <c r="E3">
         <v>9</v>
@@ -3641,10 +3827,10 @@
         <v>1080</v>
       </c>
       <c r="G3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -3696,12 +3882,12 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B6" t="s">
         <v>116</v>
@@ -3722,12 +3908,12 @@
         <v>15</v>
       </c>
       <c r="H6" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B7" t="s">
         <v>55</v>
@@ -3745,15 +3931,15 @@
         <v>285</v>
       </c>
       <c r="G7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B8" t="s">
         <v>48</v>
@@ -3779,7 +3965,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B9" t="s">
         <v>124</v>
@@ -3805,7 +3991,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
@@ -3826,12 +4012,12 @@
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B11" t="s">
         <v>80</v>
@@ -3852,12 +4038,12 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B12" t="s">
         <v>59</v>
@@ -3883,7 +4069,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B13" t="s">
         <v>139</v>
@@ -3909,10 +4095,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C14" t="s">
         <v>23</v>
@@ -3935,10 +4121,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
@@ -3961,10 +4147,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
@@ -3987,10 +4173,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
@@ -4008,15 +4194,15 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C18" t="s">
         <v>18</v>
@@ -4039,10 +4225,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B19" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
@@ -4060,15 +4246,15 @@
         <v>15</v>
       </c>
       <c r="H19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -4091,10 +4277,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C21" t="s">
         <v>117</v>
@@ -4117,10 +4303,10 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B22" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C22" t="s">
         <v>117</v>
@@ -4143,10 +4329,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B23" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -4169,10 +4355,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B24" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C24" t="s">
         <v>29</v>
@@ -4195,10 +4381,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B25" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C25" t="s">
         <v>26</v>
@@ -4221,10 +4407,10 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B26" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C26" t="s">
         <v>23</v>
@@ -4242,15 +4428,15 @@
         <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B27" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C27" t="s">
         <v>23</v>
@@ -4273,10 +4459,10 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B28" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C28" t="s">
         <v>23</v>
@@ -4294,15 +4480,15 @@
         <v>15</v>
       </c>
       <c r="H28" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B29" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C29" t="s">
         <v>23</v>
@@ -4320,15 +4506,15 @@
         <v>15</v>
       </c>
       <c r="H29" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C30" t="s">
         <v>23</v>
@@ -4351,10 +4537,10 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B31" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C31" t="s">
         <v>60</v>
@@ -4377,10 +4563,10 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C32" t="s">
         <v>18</v>
@@ -4398,15 +4584,15 @@
         <v>15</v>
       </c>
       <c r="H32" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C33" t="s">
         <v>29</v>
@@ -4429,10 +4615,10 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B34" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C34" t="s">
         <v>29</v>
@@ -4450,15 +4636,15 @@
         <v>15</v>
       </c>
       <c r="H34" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B35" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C35" t="s">
         <v>60</v>
@@ -4481,10 +4667,10 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C36" t="s">
         <v>23</v>
@@ -4507,10 +4693,10 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B37" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C37" t="s">
         <v>26</v>
@@ -4533,10 +4719,10 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B38" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C38" t="s">
         <v>23</v>
@@ -4554,15 +4740,15 @@
         <v>15</v>
       </c>
       <c r="H38" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B39" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C39" t="s">
         <v>117</v>
@@ -4577,18 +4763,18 @@
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H39" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C40" t="s">
         <v>23</v>
@@ -4603,10 +4789,556 @@
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H40" t="s">
-        <v>184</v>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>258</v>
+      </c>
+      <c r="B41" t="s">
+        <v>259</v>
+      </c>
+      <c r="C41" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41">
+        <v>10</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41" t="s">
+        <v>260</v>
+      </c>
+      <c r="H41" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>261</v>
+      </c>
+      <c r="B42" t="s">
+        <v>262</v>
+      </c>
+      <c r="C42" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42">
+        <v>10</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42" t="s">
+        <v>263</v>
+      </c>
+      <c r="H42" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>264</v>
+      </c>
+      <c r="B43" t="s">
+        <v>265</v>
+      </c>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43">
+        <v>10</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43" t="s">
+        <v>266</v>
+      </c>
+      <c r="H43" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>267</v>
+      </c>
+      <c r="B44" t="s">
+        <v>268</v>
+      </c>
+      <c r="C44" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44">
+        <v>10</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44" t="s">
+        <v>269</v>
+      </c>
+      <c r="H44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>270</v>
+      </c>
+      <c r="B45" t="s">
+        <v>271</v>
+      </c>
+      <c r="C45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45">
+        <v>10</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45" t="s">
+        <v>272</v>
+      </c>
+      <c r="H45" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>273</v>
+      </c>
+      <c r="B46" t="s">
+        <v>274</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46">
+        <v>10</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46" t="s">
+        <v>275</v>
+      </c>
+      <c r="H46" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>276</v>
+      </c>
+      <c r="B47" t="s">
+        <v>277</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47">
+        <v>10</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47" t="s">
+        <v>278</v>
+      </c>
+      <c r="H47" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>279</v>
+      </c>
+      <c r="B48" t="s">
+        <v>280</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48">
+        <v>10</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48" t="s">
+        <v>281</v>
+      </c>
+      <c r="H48" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>282</v>
+      </c>
+      <c r="B49" t="s">
+        <v>283</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49">
+        <v>10</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49" t="s">
+        <v>284</v>
+      </c>
+      <c r="H49" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>285</v>
+      </c>
+      <c r="B50" t="s">
+        <v>286</v>
+      </c>
+      <c r="C50" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50">
+        <v>10</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50" t="s">
+        <v>287</v>
+      </c>
+      <c r="H50" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>288</v>
+      </c>
+      <c r="B51" t="s">
+        <v>289</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>10</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51" t="s">
+        <v>290</v>
+      </c>
+      <c r="H51" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>291</v>
+      </c>
+      <c r="B52" t="s">
+        <v>292</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>10</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52" t="s">
+        <v>293</v>
+      </c>
+      <c r="H52" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>294</v>
+      </c>
+      <c r="B53" t="s">
+        <v>295</v>
+      </c>
+      <c r="C53" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53">
+        <v>10</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53" t="s">
+        <v>296</v>
+      </c>
+      <c r="H53" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>297</v>
+      </c>
+      <c r="B54" t="s">
+        <v>295</v>
+      </c>
+      <c r="C54" t="s">
+        <v>26</v>
+      </c>
+      <c r="D54">
+        <v>10</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54" t="s">
+        <v>298</v>
+      </c>
+      <c r="H54" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>299</v>
+      </c>
+      <c r="B55" t="s">
+        <v>295</v>
+      </c>
+      <c r="C55" t="s">
+        <v>26</v>
+      </c>
+      <c r="D55">
+        <v>10</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55" t="s">
+        <v>300</v>
+      </c>
+      <c r="H55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>301</v>
+      </c>
+      <c r="B56" t="s">
+        <v>302</v>
+      </c>
+      <c r="C56" t="s">
+        <v>117</v>
+      </c>
+      <c r="D56">
+        <v>10</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56" t="s">
+        <v>303</v>
+      </c>
+      <c r="H56" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>304</v>
+      </c>
+      <c r="B57" t="s">
+        <v>305</v>
+      </c>
+      <c r="C57" t="s">
+        <v>117</v>
+      </c>
+      <c r="D57">
+        <v>10</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57" t="s">
+        <v>306</v>
+      </c>
+      <c r="H57" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>307</v>
+      </c>
+      <c r="B58" t="s">
+        <v>308</v>
+      </c>
+      <c r="C58" t="s">
+        <v>117</v>
+      </c>
+      <c r="D58">
+        <v>10</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58" t="s">
+        <v>309</v>
+      </c>
+      <c r="H58" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>310</v>
+      </c>
+      <c r="B59" t="s">
+        <v>311</v>
+      </c>
+      <c r="C59" t="s">
+        <v>117</v>
+      </c>
+      <c r="D59">
+        <v>10</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59" t="s">
+        <v>312</v>
+      </c>
+      <c r="H59" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>313</v>
+      </c>
+      <c r="B60" t="s">
+        <v>314</v>
+      </c>
+      <c r="C60" t="s">
+        <v>117</v>
+      </c>
+      <c r="D60">
+        <v>10</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60" t="s">
+        <v>315</v>
+      </c>
+      <c r="H60" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>316</v>
+      </c>
+      <c r="B61" t="s">
+        <v>317</v>
+      </c>
+      <c r="C61" t="s">
+        <v>117</v>
+      </c>
+      <c r="D61">
+        <v>10</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61" t="s">
+        <v>318</v>
+      </c>
+      <c r="H61" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -4628,30 +5360,30 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>257</v>
+        <v>319</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>258</v>
+        <v>320</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>259</v>
+        <v>321</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>260</v>
+        <v>322</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>261</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>262</v>
+        <v>324</v>
       </c>
       <c r="B2">
         <v>464</v>
@@ -4674,7 +5406,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>263</v>
+        <v>325</v>
       </c>
       <c r="B3">
         <v>630</v>
@@ -4697,7 +5429,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>264</v>
+        <v>326</v>
       </c>
       <c r="B4">
         <v>1553</v>
@@ -4720,7 +5452,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>265</v>
+        <v>327</v>
       </c>
       <c r="B5">
         <v>64</v>
@@ -4743,7 +5475,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>266</v>
+        <v>328</v>
       </c>
       <c r="B6">
         <v>140</v>
@@ -4766,7 +5498,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>267</v>
+        <v>329</v>
       </c>
       <c r="B7">
         <v>170</v>
@@ -4789,7 +5521,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>268</v>
+        <v>330</v>
       </c>
       <c r="B8">
         <v>280</v>
@@ -4812,7 +5544,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>269</v>
+        <v>331</v>
       </c>
       <c r="B9">
         <v>2738</v>
@@ -4835,7 +5567,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>270</v>
+        <v>332</v>
       </c>
       <c r="B10">
         <v>1290</v>

</xml_diff>